<commit_message>
Add Excel sheet captures to case 1 and fix assumption labels in demo matrix
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QtwA9GGkLZAYr7iDv4MyAb
</commit_message>
<xml_diff>
--- a/01-tarifario-jbg/matriz_demo.xlsx
+++ b/01-tarifario-jbg/matriz_demo.xlsx
@@ -2557,7 +2557,7 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="14"/>
@@ -2576,24 +2576,24 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="s">
+      <c r="B2" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="12" t="n">
+      <c r="C2" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
+      <c r="B3" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="B3" s="12" t="n">
+      <c r="C3" s="12" t="n">
         <v>0.1</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>107</v>
       </c>
     </row>
@@ -2682,7 +2682,7 @@
         <v>A</v>
       </c>
       <c r="M6" s="10" t="str">
-        <f aca="false">IF(H6&lt;$B$2,"Margen bajo",IF(I6&lt;-$B$3,"Bajo mercado",IF(I6&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H6&lt;$C$2,"Margen bajo",IF(I6&lt;-$C$3,"Bajo mercado",IF(I6&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -2730,7 +2730,7 @@
         <v>A</v>
       </c>
       <c r="M7" s="10" t="str">
-        <f aca="false">IF(H7&lt;$B$2,"Margen bajo",IF(I7&lt;-$B$3,"Bajo mercado",IF(I7&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H7&lt;$C$2,"Margen bajo",IF(I7&lt;-$C$3,"Bajo mercado",IF(I7&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Sobre mercado</v>
       </c>
     </row>
@@ -2778,7 +2778,7 @@
         <v>A</v>
       </c>
       <c r="M8" s="10" t="str">
-        <f aca="false">IF(H8&lt;$B$2,"Margen bajo",IF(I8&lt;-$B$3,"Bajo mercado",IF(I8&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H8&lt;$C$2,"Margen bajo",IF(I8&lt;-$C$3,"Bajo mercado",IF(I8&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
         <v>A</v>
       </c>
       <c r="M9" s="10" t="str">
-        <f aca="false">IF(H9&lt;$B$2,"Margen bajo",IF(I9&lt;-$B$3,"Bajo mercado",IF(I9&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H9&lt;$C$2,"Margen bajo",IF(I9&lt;-$C$3,"Bajo mercado",IF(I9&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Bajo mercado</v>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
         <v>A</v>
       </c>
       <c r="M10" s="10" t="str">
-        <f aca="false">IF(H10&lt;$B$2,"Margen bajo",IF(I10&lt;-$B$3,"Bajo mercado",IF(I10&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H10&lt;$C$2,"Margen bajo",IF(I10&lt;-$C$3,"Bajo mercado",IF(I10&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
         <v>A</v>
       </c>
       <c r="M11" s="10" t="str">
-        <f aca="false">IF(H11&lt;$B$2,"Margen bajo",IF(I11&lt;-$B$3,"Bajo mercado",IF(I11&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H11&lt;$C$2,"Margen bajo",IF(I11&lt;-$C$3,"Bajo mercado",IF(I11&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Sobre mercado</v>
       </c>
     </row>
@@ -2970,7 +2970,7 @@
         <v>A</v>
       </c>
       <c r="M12" s="10" t="str">
-        <f aca="false">IF(H12&lt;$B$2,"Margen bajo",IF(I12&lt;-$B$3,"Bajo mercado",IF(I12&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H12&lt;$C$2,"Margen bajo",IF(I12&lt;-$C$3,"Bajo mercado",IF(I12&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
         <v>A</v>
       </c>
       <c r="M13" s="10" t="str">
-        <f aca="false">IF(H13&lt;$B$2,"Margen bajo",IF(I13&lt;-$B$3,"Bajo mercado",IF(I13&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H13&lt;$C$2,"Margen bajo",IF(I13&lt;-$C$3,"Bajo mercado",IF(I13&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3066,7 +3066,7 @@
         <v>A</v>
       </c>
       <c r="M14" s="10" t="str">
-        <f aca="false">IF(H14&lt;$B$2,"Margen bajo",IF(I14&lt;-$B$3,"Bajo mercado",IF(I14&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H14&lt;$C$2,"Margen bajo",IF(I14&lt;-$C$3,"Bajo mercado",IF(I14&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Bajo mercado</v>
       </c>
     </row>
@@ -3114,7 +3114,7 @@
         <v>A</v>
       </c>
       <c r="M15" s="10" t="str">
-        <f aca="false">IF(H15&lt;$B$2,"Margen bajo",IF(I15&lt;-$B$3,"Bajo mercado",IF(I15&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H15&lt;$C$2,"Margen bajo",IF(I15&lt;-$C$3,"Bajo mercado",IF(I15&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
         <v>B</v>
       </c>
       <c r="M16" s="10" t="str">
-        <f aca="false">IF(H16&lt;$B$2,"Margen bajo",IF(I16&lt;-$B$3,"Bajo mercado",IF(I16&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H16&lt;$C$2,"Margen bajo",IF(I16&lt;-$C$3,"Bajo mercado",IF(I16&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
         <v>B</v>
       </c>
       <c r="M17" s="10" t="str">
-        <f aca="false">IF(H17&lt;$B$2,"Margen bajo",IF(I17&lt;-$B$3,"Bajo mercado",IF(I17&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H17&lt;$C$2,"Margen bajo",IF(I17&lt;-$C$3,"Bajo mercado",IF(I17&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
         <v>B</v>
       </c>
       <c r="M18" s="10" t="str">
-        <f aca="false">IF(H18&lt;$B$2,"Margen bajo",IF(I18&lt;-$B$3,"Bajo mercado",IF(I18&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H18&lt;$C$2,"Margen bajo",IF(I18&lt;-$C$3,"Bajo mercado",IF(I18&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3306,7 +3306,7 @@
         <v>B</v>
       </c>
       <c r="M19" s="10" t="str">
-        <f aca="false">IF(H19&lt;$B$2,"Margen bajo",IF(I19&lt;-$B$3,"Bajo mercado",IF(I19&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H19&lt;$C$2,"Margen bajo",IF(I19&lt;-$C$3,"Bajo mercado",IF(I19&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
         <v>B</v>
       </c>
       <c r="M20" s="10" t="str">
-        <f aca="false">IF(H20&lt;$B$2,"Margen bajo",IF(I20&lt;-$B$3,"Bajo mercado",IF(I20&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H20&lt;$C$2,"Margen bajo",IF(I20&lt;-$C$3,"Bajo mercado",IF(I20&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3402,7 +3402,7 @@
         <v>B</v>
       </c>
       <c r="M21" s="10" t="str">
-        <f aca="false">IF(H21&lt;$B$2,"Margen bajo",IF(I21&lt;-$B$3,"Bajo mercado",IF(I21&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H21&lt;$C$2,"Margen bajo",IF(I21&lt;-$C$3,"Bajo mercado",IF(I21&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
         <v>B</v>
       </c>
       <c r="M22" s="10" t="str">
-        <f aca="false">IF(H22&lt;$B$2,"Margen bajo",IF(I22&lt;-$B$3,"Bajo mercado",IF(I22&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H22&lt;$C$2,"Margen bajo",IF(I22&lt;-$C$3,"Bajo mercado",IF(I22&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3498,7 +3498,7 @@
         <v>B</v>
       </c>
       <c r="M23" s="10" t="str">
-        <f aca="false">IF(H23&lt;$B$2,"Margen bajo",IF(I23&lt;-$B$3,"Bajo mercado",IF(I23&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H23&lt;$C$2,"Margen bajo",IF(I23&lt;-$C$3,"Bajo mercado",IF(I23&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Bajo mercado</v>
       </c>
     </row>
@@ -3546,7 +3546,7 @@
         <v>B</v>
       </c>
       <c r="M24" s="10" t="str">
-        <f aca="false">IF(H24&lt;$B$2,"Margen bajo",IF(I24&lt;-$B$3,"Bajo mercado",IF(I24&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H24&lt;$C$2,"Margen bajo",IF(I24&lt;-$C$3,"Bajo mercado",IF(I24&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3594,7 +3594,7 @@
         <v>B</v>
       </c>
       <c r="M25" s="10" t="str">
-        <f aca="false">IF(H25&lt;$B$2,"Margen bajo",IF(I25&lt;-$B$3,"Bajo mercado",IF(I25&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H25&lt;$C$2,"Margen bajo",IF(I25&lt;-$C$3,"Bajo mercado",IF(I25&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3642,7 +3642,7 @@
         <v>B</v>
       </c>
       <c r="M26" s="10" t="str">
-        <f aca="false">IF(H26&lt;$B$2,"Margen bajo",IF(I26&lt;-$B$3,"Bajo mercado",IF(I26&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H26&lt;$C$2,"Margen bajo",IF(I26&lt;-$C$3,"Bajo mercado",IF(I26&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Bajo mercado</v>
       </c>
     </row>
@@ -3690,7 +3690,7 @@
         <v>B</v>
       </c>
       <c r="M27" s="10" t="str">
-        <f aca="false">IF(H27&lt;$B$2,"Margen bajo",IF(I27&lt;-$B$3,"Bajo mercado",IF(I27&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H27&lt;$C$2,"Margen bajo",IF(I27&lt;-$C$3,"Bajo mercado",IF(I27&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
         <v>B</v>
       </c>
       <c r="M28" s="10" t="str">
-        <f aca="false">IF(H28&lt;$B$2,"Margen bajo",IF(I28&lt;-$B$3,"Bajo mercado",IF(I28&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H28&lt;$C$2,"Margen bajo",IF(I28&lt;-$C$3,"Bajo mercado",IF(I28&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Margen bajo</v>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
         <v>B</v>
       </c>
       <c r="M29" s="10" t="str">
-        <f aca="false">IF(H29&lt;$B$2,"Margen bajo",IF(I29&lt;-$B$3,"Bajo mercado",IF(I29&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H29&lt;$C$2,"Margen bajo",IF(I29&lt;-$C$3,"Bajo mercado",IF(I29&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Sobre mercado</v>
       </c>
     </row>
@@ -3834,7 +3834,7 @@
         <v>B</v>
       </c>
       <c r="M30" s="10" t="str">
-        <f aca="false">IF(H30&lt;$B$2,"Margen bajo",IF(I30&lt;-$B$3,"Bajo mercado",IF(I30&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H30&lt;$C$2,"Margen bajo",IF(I30&lt;-$C$3,"Bajo mercado",IF(I30&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3882,7 +3882,7 @@
         <v>B</v>
       </c>
       <c r="M31" s="10" t="str">
-        <f aca="false">IF(H31&lt;$B$2,"Margen bajo",IF(I31&lt;-$B$3,"Bajo mercado",IF(I31&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H31&lt;$C$2,"Margen bajo",IF(I31&lt;-$C$3,"Bajo mercado",IF(I31&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3930,7 +3930,7 @@
         <v>B</v>
       </c>
       <c r="M32" s="10" t="str">
-        <f aca="false">IF(H32&lt;$B$2,"Margen bajo",IF(I32&lt;-$B$3,"Bajo mercado",IF(I32&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H32&lt;$C$2,"Margen bajo",IF(I32&lt;-$C$3,"Bajo mercado",IF(I32&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
         <v>B</v>
       </c>
       <c r="M33" s="10" t="str">
-        <f aca="false">IF(H33&lt;$B$2,"Margen bajo",IF(I33&lt;-$B$3,"Bajo mercado",IF(I33&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H33&lt;$C$2,"Margen bajo",IF(I33&lt;-$C$3,"Bajo mercado",IF(I33&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -4026,7 +4026,7 @@
         <v>B</v>
       </c>
       <c r="M34" s="10" t="str">
-        <f aca="false">IF(H34&lt;$B$2,"Margen bajo",IF(I34&lt;-$B$3,"Bajo mercado",IF(I34&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H34&lt;$C$2,"Margen bajo",IF(I34&lt;-$C$3,"Bajo mercado",IF(I34&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Margen bajo</v>
       </c>
     </row>
@@ -4074,7 +4074,7 @@
         <v>B</v>
       </c>
       <c r="M35" s="10" t="str">
-        <f aca="false">IF(H35&lt;$B$2,"Margen bajo",IF(I35&lt;-$B$3,"Bajo mercado",IF(I35&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H35&lt;$C$2,"Margen bajo",IF(I35&lt;-$C$3,"Bajo mercado",IF(I35&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -4122,7 +4122,7 @@
         <v>B</v>
       </c>
       <c r="M36" s="10" t="str">
-        <f aca="false">IF(H36&lt;$B$2,"Margen bajo",IF(I36&lt;-$B$3,"Bajo mercado",IF(I36&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H36&lt;$C$2,"Margen bajo",IF(I36&lt;-$C$3,"Bajo mercado",IF(I36&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
         <v>B</v>
       </c>
       <c r="M37" s="10" t="str">
-        <f aca="false">IF(H37&lt;$B$2,"Margen bajo",IF(I37&lt;-$B$3,"Bajo mercado",IF(I37&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H37&lt;$C$2,"Margen bajo",IF(I37&lt;-$C$3,"Bajo mercado",IF(I37&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Bajo mercado</v>
       </c>
     </row>
@@ -4218,7 +4218,7 @@
         <v>B</v>
       </c>
       <c r="M38" s="10" t="str">
-        <f aca="false">IF(H38&lt;$B$2,"Margen bajo",IF(I38&lt;-$B$3,"Bajo mercado",IF(I38&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H38&lt;$C$2,"Margen bajo",IF(I38&lt;-$C$3,"Bajo mercado",IF(I38&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
         <v>B</v>
       </c>
       <c r="M39" s="10" t="str">
-        <f aca="false">IF(H39&lt;$B$2,"Margen bajo",IF(I39&lt;-$B$3,"Bajo mercado",IF(I39&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H39&lt;$C$2,"Margen bajo",IF(I39&lt;-$C$3,"Bajo mercado",IF(I39&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Bajo mercado</v>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
         <v>B</v>
       </c>
       <c r="M40" s="10" t="str">
-        <f aca="false">IF(H40&lt;$B$2,"Margen bajo",IF(I40&lt;-$B$3,"Bajo mercado",IF(I40&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H40&lt;$C$2,"Margen bajo",IF(I40&lt;-$C$3,"Bajo mercado",IF(I40&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Bajo mercado</v>
       </c>
     </row>
@@ -4362,7 +4362,7 @@
         <v>B</v>
       </c>
       <c r="M41" s="10" t="str">
-        <f aca="false">IF(H41&lt;$B$2,"Margen bajo",IF(I41&lt;-$B$3,"Bajo mercado",IF(I41&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H41&lt;$C$2,"Margen bajo",IF(I41&lt;-$C$3,"Bajo mercado",IF(I41&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -4410,7 +4410,7 @@
         <v>B</v>
       </c>
       <c r="M42" s="10" t="str">
-        <f aca="false">IF(H42&lt;$B$2,"Margen bajo",IF(I42&lt;-$B$3,"Bajo mercado",IF(I42&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H42&lt;$C$2,"Margen bajo",IF(I42&lt;-$C$3,"Bajo mercado",IF(I42&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>Bajo mercado</v>
       </c>
     </row>
@@ -4458,7 +4458,7 @@
         <v>B</v>
       </c>
       <c r="M43" s="10" t="str">
-        <f aca="false">IF(H43&lt;$B$2,"Margen bajo",IF(I43&lt;-$B$3,"Bajo mercado",IF(I43&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H43&lt;$C$2,"Margen bajo",IF(I43&lt;-$C$3,"Bajo mercado",IF(I43&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -4506,7 +4506,7 @@
         <v>B</v>
       </c>
       <c r="M44" s="10" t="str">
-        <f aca="false">IF(H44&lt;$B$2,"Margen bajo",IF(I44&lt;-$B$3,"Bajo mercado",IF(I44&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H44&lt;$C$2,"Margen bajo",IF(I44&lt;-$C$3,"Bajo mercado",IF(I44&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>
@@ -4554,7 +4554,7 @@
         <v>B</v>
       </c>
       <c r="M45" s="10" t="str">
-        <f aca="false">IF(H45&lt;$B$2,"Margen bajo",IF(I45&lt;-$B$3,"Bajo mercado",IF(I45&gt;$B$3,"Sobre mercado","OK")))</f>
+        <f aca="false">IF(H45&lt;$C$2,"Margen bajo",IF(I45&lt;-$C$3,"Bajo mercado",IF(I45&gt;$C$3,"Sobre mercado","OK")))</f>
         <v>OK</v>
       </c>
     </row>

</xml_diff>